<commit_message>
Optimize day routes by real driving distance; add dog-themed branding
Day clustering and stop ordering now use an OSRM driving-distance
matrix (capacitated k-medoids) instead of straight-line haversine,
cutting total driving distance by ~19km across the week. Also adds
dog-themed touches to the driver site (paw icon, PAW-01 brand mark,
paw-print background texture, paw flourishes) since the branches
distribute dog products.
</commit_message>
<xml_diff>
--- a/branches_with_waze_links_v3_days.xlsx
+++ b/branches_with_waze_links_v3_days.xlsx
@@ -442,7 +442,7 @@
     <col width="42" customWidth="1" min="4" max="4"/>
     <col width="46" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -478,7 +478,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Leg distance from previous stop (m)</t>
+          <t>Leg driving distance from previous stop (m)</t>
         </is>
       </c>
     </row>
@@ -491,22 +491,22 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי לוד</t>
+          <t>רמי לוי יבנה</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי – לוד</t>
+          <t>רמי לוי – יבנה</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.945270,34.892120&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.885700,34.733740&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>31.945270, 34.892120</t>
+          <t>31.885700, 34.733740</t>
         </is>
       </c>
       <c r="G2" s="2" t="n"/>
@@ -520,26 +520,26 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>יוחננוף רמלה</t>
+          <t>מחסני השוק יבנה</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>יוחננוף – רמלה</t>
+          <t>מחסני השוק – יבנה</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.937330,34.886180&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.877970,34.736400&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>31.937330, 34.886180</t>
+          <t>31.877970, 34.736400</t>
         </is>
       </c>
       <c r="G3" s="2" t="n">
-        <v>1046</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="4">
@@ -551,26 +551,26 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>שוק העיר רמלה רחוב דני מס</t>
+          <t>סופר בונוס יבנה</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>שוק העיר – רמלה, קניון הרמבלס</t>
+          <t>סופר בונוס – יבנה</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.929320,34.867530&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.863087,34.739125&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>31.929320, 34.867530</t>
+          <t>31.863087, 34.739125</t>
         </is>
       </c>
       <c r="G4" s="2" t="n">
-        <v>1972</v>
+        <v>2490</v>
       </c>
     </row>
     <row r="5">
@@ -582,26 +582,26 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>קרפור קלוזנר רמלה</t>
+          <t>יוחננוף עקרון</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>קרפור – קלוזנר רמלה</t>
+          <t>יוחננוף – קריית עקרון</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.919071,34.869466&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.860190,34.814490&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>31.919071, 34.869466</t>
+          <t>31.860190, 34.814490</t>
         </is>
       </c>
       <c r="G5" s="2" t="n">
-        <v>1154</v>
+        <v>10393</v>
       </c>
     </row>
     <row r="6">
@@ -613,26 +613,26 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>שוק העיר רמלה רחוב יעקב דורי</t>
+          <t>קרפור קלוזנר רמלה</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>שוק העיר – נאות שמיר, רמלה</t>
+          <t>קרפור – קלוזנר רמלה</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.929080,34.849320&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.919071,34.869466&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>31.929080, 34.849320</t>
+          <t>31.919071, 34.869466</t>
         </is>
       </c>
       <c r="G6" s="2" t="n">
-        <v>2203</v>
+        <v>9561</v>
       </c>
     </row>
     <row r="7">
@@ -644,26 +644,26 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>יוחננוף עקרון</t>
+          <t>שוק העיר רמלה רחוב יעקב דורי</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>יוחננוף – קריית עקרון</t>
+          <t>שוק העיר – נאות שמיר, רמלה</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.860190,34.814490&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.929080,34.849320&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>31.860190, 34.814490</t>
+          <t>31.929080, 34.849320</t>
         </is>
       </c>
       <c r="G7" s="2" t="n">
-        <v>8336</v>
+        <v>4145</v>
       </c>
     </row>
     <row r="8">
@@ -675,86 +675,88 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>שפע ברכה גדרה</t>
+          <t>שוק העיר רמלה רחוב דני מס</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>שפע ברכה – גדרה</t>
+          <t>שוק העיר – רמלה, קניון הרמבלס</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.818301,34.775800&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.929320,34.867530&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>31.818301, 34.775800</t>
+          <t>31.929320, 34.867530</t>
         </is>
       </c>
       <c r="G8" s="2" t="n">
-        <v>5921</v>
+        <v>2370</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B9" s="2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי יבנה</t>
+          <t>יוחננוף רמלה</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי – יבנה</t>
+          <t>יוחננוף – רמלה</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.885700,34.733740&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.937330,34.886180&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>31.885700, 34.733740</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="n"/>
+          <t>31.937330, 34.886180</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>3014</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B10" s="2" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק יבנה</t>
+          <t>רמי לוי לוד</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – יבנה</t>
+          <t>רמי לוי – לוד</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.877970,34.736400&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.945270,34.892120&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>31.877970, 34.736400</t>
+          <t>31.945270, 34.892120</t>
         </is>
       </c>
       <c r="G10" s="2" t="n">
-        <v>895</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="11">
@@ -762,61 +764,59 @@
         <v>2</v>
       </c>
       <c r="B11" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>פרש מרקט מחסני להב יבנה</t>
+          <t>מחסני השוק יד בנימין</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>מחסני להב / פרשמרקט – יבנה</t>
+          <t>מחסני השוק – יד בנימין</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.866399,34.735819&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.792720,34.824080&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>31.866399, 34.735819</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="n">
-        <v>1288</v>
-      </c>
+          <t>31.792720, 34.824080</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
         <v>2</v>
       </c>
       <c r="B12" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>סופר בונוס יבנה</t>
+          <t>מחסני הושק יד בנימין</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>סופר בונוס – יבנה</t>
+          <t>מחסני השוק – יד בנימין</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.863087,34.739125&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.792720,34.824080&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>31.863087, 34.739125</t>
+          <t>31.792720, 34.824080</t>
         </is>
       </c>
       <c r="G12" s="2" t="n">
-        <v>483</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -824,30 +824,30 @@
         <v>2</v>
       </c>
       <c r="B13" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>יוחננוף גן יבנה</t>
+          <t xml:space="preserve">יוחננוף גדרה </t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>יוחננוף – גן יבנה</t>
+          <t>יוחננוף – גדרה</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.794680,34.705580&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.797160,34.767740&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>31.794680, 34.705580</t>
+          <t>31.797160, 34.767740</t>
         </is>
       </c>
       <c r="G13" s="2" t="n">
-        <v>8240</v>
+        <v>6945</v>
       </c>
     </row>
     <row r="14">
@@ -855,30 +855,30 @@
         <v>2</v>
       </c>
       <c r="B14" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>קשת טעמים אשדוד</t>
+          <t>הסל שלנו גדרה</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>קשת טעמים – אשדוד</t>
+          <t>הסל שלנו – גדרה</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.812130,34.661190&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.800510,34.783400&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>31.812130, 34.661190</t>
+          <t>31.800510, 34.783400</t>
         </is>
       </c>
       <c r="G14" s="2" t="n">
-        <v>4622</v>
+        <v>2514</v>
       </c>
     </row>
     <row r="15">
@@ -886,152 +886,154 @@
         <v>2</v>
       </c>
       <c r="B15" s="2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי אשדוד</t>
+          <t>סיטי מרקט סניף שני גדרה</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי – אשדוד</t>
+          <t>סיטי מרקט – גדרה, סניף צהלה</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.814770,34.660040&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.800019,34.789253&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>31.814770, 34.660040</t>
+          <t>31.800019, 34.789253</t>
         </is>
       </c>
       <c r="G15" s="2" t="n">
-        <v>313</v>
+        <v>577</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B16" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">יוחננוף גדרה </t>
+          <t>סיטי מרקט סניף ראשון גדרה</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>יוחננוף – גדרה</t>
+          <t>סיטי מרקט – גדרה, סניף ציונה</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.797160,34.767740&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.804598,34.790889&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>31.797160, 34.767740</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="n"/>
+          <t>31.804598, 34.790889</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>573</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B17" s="2" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>הסל שלנו גדרה</t>
+          <t>מחסני השוק גדרה</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>הסל שלנו – גדרה</t>
+          <t>מחסני השוק – גדרה</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.800510,34.783400&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.803660,34.784850&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>31.800510, 34.783400</t>
+          <t>31.803660, 34.784850</t>
         </is>
       </c>
       <c r="G17" s="2" t="n">
-        <v>1526</v>
+        <v>833</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B18" s="2" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק גדרה</t>
+          <t>שפע ברכה גדרה</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – גדרה</t>
+          <t>שפע ברכה – גדרה</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.803660,34.784850&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.818301,34.775800&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>31.803660, 34.784850</t>
+          <t>31.818301, 34.775800</t>
         </is>
       </c>
       <c r="G18" s="2" t="n">
-        <v>376</v>
+        <v>2289</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B19" s="2" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>סיטי מרקט סניף ראשון גדרה</t>
+          <t>פרש מרקט מחסני להב יבנה</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>סיטי מרקט – גדרה, סניף ציונה</t>
+          <t>מחסני להב / פרשמרקט – יבנה</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.804598,34.790889&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.866399,34.735819&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>31.804598, 34.790889</t>
+          <t>31.866399, 34.735819</t>
         </is>
       </c>
       <c r="G19" s="2" t="n">
-        <v>580</v>
+        <v>12412</v>
       </c>
     </row>
     <row r="20">
@@ -1039,61 +1041,59 @@
         <v>3</v>
       </c>
       <c r="B20" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>סיטי מרקט סניף שני גדרה</t>
+          <t>סופר קופיקס אשדוד</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>סיטי מרקט – גדרה, סניף צהלה</t>
+          <t>סופר קופיקס – אשדוד</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.800019,34.789253&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.777726,34.636456&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>31.800019, 34.789253</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="n">
-        <v>532</v>
-      </c>
+          <t>31.777726, 34.636456</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
         <v>3</v>
       </c>
       <c r="B21" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>מחסני הושק יד בנימין</t>
+          <t>זול ובגדול אשדוד</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – יד בנימין</t>
+          <t>זול ובגדול – אשדוד</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.792720,34.824080&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.780820,34.631780&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>31.792720, 34.824080</t>
+          <t>31.780820, 34.631780</t>
         </is>
       </c>
       <c r="G21" s="2" t="n">
-        <v>3390</v>
+        <v>719</v>
       </c>
     </row>
     <row r="22">
@@ -1101,214 +1101,216 @@
         <v>3</v>
       </c>
       <c r="B22" s="2" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק יד בנימין</t>
+          <t>טסה שוקולד רחוב הציונות אשדוד</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – יד בנימין</t>
+          <t>טסה – שדרות הציונות, אשדוד</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.792720,34.824080&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.787595,34.643303&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>31.792720, 34.824080</t>
+          <t>31.787595, 34.643303</t>
         </is>
       </c>
       <c r="G22" s="2" t="n">
-        <v>0</v>
+        <v>1712</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B23" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B23" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>פרש מרקט מחסני להב רחוב גיא אוני אשדוד</t>
+          <t>קרפור ד רוגזין אשדוד</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>מחסני להב / פרשמרקט – גיא אוני</t>
+          <t>קרפור – אשדוד רובע ד׳</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.785248,34.659107&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.800290,34.641557&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>31.785248, 34.659107</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="n"/>
+          <t>31.800290, 34.641557</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>1822</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B24" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>קרפור ח אשדוד מרכז כלניות</t>
+          <t>טסה שוקולד רחוב רוגזין אשדוד</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>קרפור – אשדוד רובע ח׳, מרכז כלניות</t>
+          <t>טסה – רוגוזין, אשדוד  (client 1)</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.783685,34.653253&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.803469,34.642244&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>31.783685, 34.653253</t>
+          <t>31.803469, 34.642244</t>
         </is>
       </c>
       <c r="G24" s="2" t="n">
-        <v>580</v>
+        <v>521</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B25" s="2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>טסה שוקולד רחוב הציונות אשדוד</t>
+          <t>טסה שוקולד רחוב רוגזין אשדוד</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>טסה – שדרות הציונות, אשדוד</t>
+          <t>טסה – רוגוזין, אשדוד  (client 2)</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.787595,34.643303&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.806300,34.643792&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>31.787595, 34.643303</t>
+          <t>31.806300, 34.643792</t>
         </is>
       </c>
       <c r="G25" s="2" t="n">
-        <v>1036</v>
+        <v>351</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B26" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>קרפור ד רוגזין אשדוד</t>
+          <t>טיב טעם אשדוד</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>קרפור – אשדוד רובע ד׳</t>
+          <t>טיב טעם – אשדוד</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.800290,34.641557&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.810210,34.656140&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>31.800290, 34.641557</t>
+          <t>31.810210, 34.656140</t>
         </is>
       </c>
       <c r="G26" s="2" t="n">
-        <v>1421</v>
+        <v>1843</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B27" s="2" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>טסה שוקולד רחוב רוגזין אשדוד</t>
+          <t>קשת טעמים אשדוד</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>טסה – רוגוזין, אשדוד  (client 1)</t>
+          <t>קשת טעמים – אשדוד</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.803469,34.642244&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.812130,34.661190&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>31.803469, 34.642244</t>
+          <t>31.812130, 34.661190</t>
         </is>
       </c>
       <c r="G27" s="2" t="n">
-        <v>359</v>
+        <v>996</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B28" s="2" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>טסה שוקולד רחוב רוגזין אשדוד</t>
+          <t>רמי לוי אשדוד</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>טסה – רוגוזין, אשדוד  (client 2)</t>
+          <t>רמי לוי – אשדוד</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.806300,34.643792&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.814770,34.660040&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>31.806300, 34.643792</t>
+          <t>31.814770, 34.660040</t>
         </is>
       </c>
       <c r="G28" s="2" t="n">
-        <v>347</v>
+        <v>924</v>
       </c>
     </row>
     <row r="29">
@@ -1316,245 +1318,245 @@
         <v>4</v>
       </c>
       <c r="B29" s="2" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>טיב טעם אשדוד</t>
+          <t>יוחננוף גן יבנה</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>טיב טעם – אשדוד</t>
+          <t>יוחננוף – גן יבנה</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.810210,34.656140&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.794680,34.705580&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>31.810210, 34.656140</t>
-        </is>
-      </c>
-      <c r="G29" s="2" t="n">
-        <v>1245</v>
-      </c>
+          <t>31.794680, 34.705580</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B30" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>קרפור אשקלון בסיטי קיבוץ גלויות 5</t>
+          <t>קרפור ח אשדוד מרכז כלניות</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>קרפור – אשקלון סיטי</t>
+          <t>קרפור – אשדוד רובע ח׳, מרכז כלניות</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.655189,34.556142&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.783685,34.653253&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>31.655189, 34.556142</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="n"/>
+          <t>31.783685, 34.653253</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>6294</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B31" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>שוק העיר מכללה אשקלון רחוב אלי כהן</t>
+          <t>פרש מרקט מחסני להב רחוב שהם אשדוד</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>שוק העיר – מכללה אשקלון</t>
+          <t>מחסני להב / פרשמרקט – שוהם</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.667450,34.569030&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.766695,34.631168&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>31.667450, 34.569030</t>
+          <t>31.766695, 34.631168</t>
         </is>
       </c>
       <c r="G31" s="2" t="n">
-        <v>1829</v>
+        <v>3633</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B32" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי אשקלון צפון</t>
+          <t>פרש מרקט מחסני להב רחוב גיא אוני אשדוד</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי – אשקלון צפון</t>
+          <t>מחסני להב / פרשמרקט – גיא אוני</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.662130,34.594590&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.785248,34.659107&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>31.662130, 34.594590</t>
+          <t>31.785248, 34.659107</t>
         </is>
       </c>
       <c r="G32" s="2" t="n">
-        <v>2490</v>
+        <v>4259</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B33" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B33" s="2" t="n">
-        <v>4</v>
-      </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>קרפור אפרידר שדרות ירושלים</t>
+          <t>יוחננוף מבקיעים אשקלון</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>קרפור – אפרידר</t>
+          <t>יוחננוף – מבקיעים</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.677410,34.575410&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.701280,34.579940&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>31.677410, 34.575410</t>
+          <t>31.701280, 34.579940</t>
         </is>
       </c>
       <c r="G33" s="2" t="n">
-        <v>2486</v>
+        <v>16150</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B34" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>יוחננוף מבקיעים אשקלון</t>
+          <t>קרפור אפרידר שדרות ירושלים</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>יוחננוף – מבקיעים</t>
+          <t>קרפור – אפרידר</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.701280,34.579940&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.677410,34.575410&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>31.701280, 34.579940</t>
+          <t>31.677410, 34.575410</t>
         </is>
       </c>
       <c r="G34" s="2" t="n">
-        <v>2689</v>
+        <v>2994</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B35" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>פרש מרקט מחסני להב רחוב שהם אשדוד</t>
+          <t>שוק העיר מכללה אשקלון רחוב אלי כהן</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>מחסני להב / פרשמרקט – שוהם</t>
+          <t>שוק העיר – מכללה אשקלון</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.766695,34.631168&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.667450,34.569030&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>31.766695, 34.631168</t>
+          <t>31.667450, 34.569030</t>
         </is>
       </c>
       <c r="G35" s="2" t="n">
-        <v>8740</v>
+        <v>1716</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B36" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>סופר קופיקס אשדוד</t>
+          <t>קרפור אשקלון בסיטי קיבוץ גלויות 5</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>סופר קופיקס – אשדוד</t>
+          <t>קרפור – אשקלון סיטי</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.777726,34.636456&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.655189,34.556142&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>31.777726, 34.636456</t>
+          <t>31.655189, 34.556142</t>
         </is>
       </c>
       <c r="G36" s="2" t="n">
-        <v>1325</v>
+        <v>2276</v>
       </c>
     </row>
     <row r="37">
@@ -1562,38 +1564,36 @@
         <v>5</v>
       </c>
       <c r="B37" s="2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>זול ובגדול אשדוד</t>
+          <t>מחסני השוק קרית מלאכי</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>זול ובגדול – אשדוד</t>
+          <t>מחסני השוק – קריית מלאכי</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.780820,34.631780&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.731658,34.753038&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>31.780820, 34.631780</t>
-        </is>
-      </c>
-      <c r="G37" s="2" t="n">
-        <v>560</v>
-      </c>
+          <t>31.731658, 34.753038</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B38" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
@@ -1615,161 +1615,163 @@
           <t>31.731658, 34.753038</t>
         </is>
       </c>
-      <c r="G38" s="2" t="n"/>
+      <c r="G38" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B39" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק קרית מלאכי</t>
+          <t>רמי לוי קסטינה</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – קריית מלאכי</t>
+          <t>רמי לוי – קסטינה</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.731658,34.753038&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.727796,34.754099&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>31.731658, 34.753038</t>
+          <t>31.727796, 34.754099</t>
         </is>
       </c>
       <c r="G39" s="2" t="n">
-        <v>0</v>
+        <v>1045</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B40" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי קסטינה</t>
+          <t>רמי לוי כרמי גת- בוייז ספורטק קריית גת</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי – קסטינה</t>
+          <t>רמי לוי כרמי גת / סופרמרקט בקריית גת</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.727796,34.754099&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.626950,34.771360&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>31.727796, 34.754099</t>
+          <t>31.626950, 34.771360</t>
         </is>
       </c>
       <c r="G40" s="2" t="n">
-        <v>441</v>
+        <v>16232</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B41" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי כרמי גת- בוייז ספורטק קריית גת</t>
+          <t>שוק העיר קריית גת- עבודה פרש סוללות ופזים</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי כרמי גת / סופרמרקט בקריית גת</t>
+          <t>שוק העיר – קריית גת / הערת עבודה נוספת</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.626950,34.771360&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.604380,34.774310&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>31.626950, 34.771360</t>
+          <t>31.604380, 34.774310</t>
         </is>
       </c>
       <c r="G41" s="2" t="n">
-        <v>11332</v>
+        <v>3318</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B42" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B42" s="2" t="n">
-        <v>5</v>
-      </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>שוק העיר קריית גת- עבודה פרש סוללות ופזים</t>
+          <t>רמי לוי קריית גת</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>שוק העיר – קריית גת / הערת עבודה נוספת</t>
+          <t>רמי לוי – קריית גת</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.604380,34.774310&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.603820,34.772470&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>31.604380, 34.774310</t>
+          <t>31.603820, 34.772470</t>
         </is>
       </c>
       <c r="G42" s="2" t="n">
-        <v>2525</v>
+        <v>293</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B43" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי קריית גת</t>
+          <t>מחסני השוק קריית גת</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי – קריית גת</t>
+          <t>מחסני השוק – קריית גת</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.603820,34.772470&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.601807,34.772956&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>31.603820, 34.772470</t>
+          <t>31.601807, 34.772956</t>
         </is>
       </c>
       <c r="G43" s="2" t="n">
-        <v>185</v>
+        <v>554</v>
       </c>
     </row>
     <row r="44">
@@ -1777,98 +1779,98 @@
         <v>6</v>
       </c>
       <c r="B44" s="2" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק קריית גת</t>
+          <t>יוחננוף נתיבות רחוב אליהו אילוז</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – קריית גת</t>
+          <t>יוחננוף – נתיבות, אליהו אילוז</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.601807,34.772956&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.412450,34.572680&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>31.601807, 34.772956</t>
-        </is>
-      </c>
-      <c r="G44" s="2" t="n">
-        <v>229</v>
-      </c>
+          <t>31.412450, 34.572680</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B45" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי שדרות</t>
+          <t>קרפור נתיבות</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי – שדרות</t>
+          <t>קרפור – נתיבות</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.526502,34.602092&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.417980,34.592430&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>31.526502, 34.602092</t>
-        </is>
-      </c>
-      <c r="G45" s="2" t="n"/>
+          <t>31.417980, 34.592430</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="n">
+        <v>2656</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B46" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>קרפור שדרות</t>
+          <t>יוחננוף נתיבות רחוב בעלי המלאכה</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>קרפור – שדרות</t>
+          <t>יוחננוף – נתיבות, בעלי המלאכה</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.523700,34.605850&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.418300,34.597040&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>31.523700, 34.605850</t>
+          <t>31.418300, 34.597040</t>
         </is>
       </c>
       <c r="G46" s="2" t="n">
-        <v>473</v>
+        <v>449</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B47" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
@@ -1891,100 +1893,100 @@
         </is>
       </c>
       <c r="G47" s="2" t="n">
-        <v>11911</v>
+        <v>2710</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B48" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>יוחננוף נתיבות רחוב בעלי המלאכה</t>
+          <t>קרפור שדרות</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>יוחננוף – נתיבות, בעלי המלאכה</t>
+          <t>קרפור – שדרות</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.418300,34.597040&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.523700,34.605850&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>31.418300, 34.597040</t>
+          <t>31.523700, 34.605850</t>
         </is>
       </c>
       <c r="G48" s="2" t="n">
-        <v>1769</v>
+        <v>14390</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B49" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>קרפור נתיבות</t>
+          <t>רמי לוי שדרות</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>קרפור – נתיבות</t>
+          <t>רמי לוי – שדרות</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.417980,34.592430&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.526502,34.602092&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>31.417980, 34.592430</t>
+          <t>31.526502, 34.602092</t>
         </is>
       </c>
       <c r="G49" s="2" t="n">
-        <v>439</v>
+        <v>904</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B50" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B50" s="2" t="n">
-        <v>6</v>
-      </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>יוחננוף נתיבות רחוב אליהו אילוז</t>
+          <t>רמי לוי אשקלון צפון</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>יוחננוף – נתיבות, אליהו אילוז</t>
+          <t>רמי לוי – אשקלון צפון</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.412450,34.572680&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.662130,34.594590&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>31.412450, 34.572680</t>
+          <t>31.662130, 34.594590</t>
         </is>
       </c>
       <c r="G50" s="2" t="n">
-        <v>1972</v>
+        <v>20709</v>
       </c>
     </row>
     <row r="51">
@@ -1992,61 +1994,59 @@
         <v>7</v>
       </c>
       <c r="B51" s="2" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק אופקים</t>
+          <t>רמי לוי ביג ב״ש</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – אופקים, מבנה</t>
+          <t>רמי לוי – BIG באר שבע</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.315153,34.624786&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.242737,34.813938&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>31.315153, 34.624786</t>
-        </is>
-      </c>
-      <c r="G51" s="2" t="n">
-        <v>11896</v>
-      </c>
+          <t>31.242737, 34.813938</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
         <v>7</v>
       </c>
       <c r="B52" s="2" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי אופקים</t>
+          <t>טיב טעם ב״ש</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי – אופקים</t>
+          <t>טיב טעם – באר שבע</t>
         </is>
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.293210,34.612890&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.247910,34.812220&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>31.293210, 34.612890</t>
+          <t>31.247910, 34.812220</t>
         </is>
       </c>
       <c r="G52" s="2" t="n">
-        <v>2689</v>
+        <v>920</v>
       </c>
     </row>
     <row r="53">
@@ -2054,152 +2054,154 @@
         <v>7</v>
       </c>
       <c r="B53" s="2" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק הקריה החרדית</t>
+          <t>מחסני השוק האורגים</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק מהדרין – הקריה החרדית</t>
+          <t>מחסני השוק – האורגים</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.267940,34.778430&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.254180,34.817730&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>31.267940, 34.778430</t>
+          <t>31.254180, 34.817730</t>
         </is>
       </c>
       <c r="G53" s="2" t="n">
-        <v>15980</v>
+        <v>1457</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B54" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>קרפור נווה זאב ב״ש</t>
+          <t>ח.נ משקאות הסיטונאי</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>קרפור – נווה זאב</t>
+          <t>ח.נ משקאות הסיטונאי</t>
         </is>
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.239300,34.773840&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.255990,34.816697&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>31.239300, 34.773840</t>
-        </is>
-      </c>
-      <c r="G54" s="2" t="n"/>
+          <t>31.255990, 34.816697</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="n">
+        <v>594</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B55" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק שכונה ט</t>
+          <t>מחסני השוק מיתרים</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – שכונה ט׳</t>
+          <t>מחסני השוק – מיתרים</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.245847,34.780029&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.374910,35.007250&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>31.245847, 34.780029</t>
+          <t>31.374910, 35.007250</t>
         </is>
       </c>
       <c r="G55" s="2" t="n">
-        <v>936</v>
+        <v>24366</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B56" s="2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק יעלים</t>
+          <t>קרפור ערד</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – יעלים</t>
+          <t>קרפור – ערד</t>
         </is>
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.251100,34.779480&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.248230,35.201160&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>31.251100, 34.779480</t>
+          <t>31.248230, 35.201160</t>
         </is>
       </c>
       <c r="G56" s="2" t="n">
-        <v>586</v>
+        <v>34289</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B57" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>מחסני להב ב״ש</t>
+          <t>מחסני השוק ערד</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>מחסני להב – באר שבע</t>
+          <t>מחסני השוק – ערד</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.250485,34.771336&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.248640,35.199280&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>31.250485, 34.771336</t>
+          <t>31.248640, 35.199280</t>
         </is>
       </c>
       <c r="G57" s="2" t="n">
-        <v>777</v>
+        <v>525</v>
       </c>
     </row>
     <row r="58">
@@ -2207,61 +2209,59 @@
         <v>8</v>
       </c>
       <c r="B58" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק רד״ק</t>
+          <t>מחסני השוק רמות</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – רד״ק</t>
+          <t>מחסני השוק – רמות</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.256575,34.771383&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.280323,34.804813&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>31.256575, 34.771383</t>
-        </is>
-      </c>
-      <c r="G58" s="2" t="n">
-        <v>677</v>
-      </c>
+          <t>31.280323, 34.804813</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
         <v>8</v>
       </c>
       <c r="B59" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק עובדה</t>
+          <t>קרפור צפון ב״ש רחוב אברהם אבינו</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – עובדה</t>
+          <t>קרפור – באר שבע, שכונה ד׳</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.259650,34.780120&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.270018,34.797222&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>31.259650, 34.780120</t>
+          <t>31.270018, 34.797222</t>
         </is>
       </c>
       <c r="G59" s="2" t="n">
-        <v>898</v>
+        <v>2412</v>
       </c>
     </row>
     <row r="60">
@@ -2269,30 +2269,30 @@
         <v>8</v>
       </c>
       <c r="B60" s="2" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>קרפור קניון אביה</t>
+          <t>מחסני השוק הקריה החרדית</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>קרפור – קניון אביה</t>
+          <t>מחסני השוק מהדרין – הקריה החרדית</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.263278,34.778719&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.267940,34.778430&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>31.263278, 34.778719</t>
+          <t>31.267940, 34.778430</t>
         </is>
       </c>
       <c r="G60" s="2" t="n">
-        <v>425</v>
+        <v>2175</v>
       </c>
     </row>
     <row r="61">
@@ -2300,30 +2300,30 @@
         <v>8</v>
       </c>
       <c r="B61" s="2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>קרפור צפון ב״ש רחוב אברהם אבינו</t>
+          <t>קרפור קניון אביה</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>קרפור – באר שבע, שכונה ד׳</t>
+          <t>קרפור – קניון אביה</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.270018,34.797222&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.263278,34.778719&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>31.270018, 34.797222</t>
+          <t>31.263278, 34.778719</t>
         </is>
       </c>
       <c r="G61" s="2" t="n">
-        <v>1912</v>
+        <v>927</v>
       </c>
     </row>
     <row r="62">
@@ -2331,90 +2331,92 @@
         <v>8</v>
       </c>
       <c r="B62" s="2" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק רמות</t>
+          <t>מחסני השוק עובדה</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – רמות</t>
+          <t>מחסני השוק – עובדה</t>
         </is>
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.280323,34.804813&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.259650,34.780120&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>31.280323, 34.804813</t>
+          <t>31.259650, 34.780120</t>
         </is>
       </c>
       <c r="G62" s="2" t="n">
-        <v>1354</v>
+        <v>948</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B63" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>קשת טעמים ב״ש</t>
+          <t>מחסני השוק רד״ק</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>קשת טעמים – באר שבע</t>
+          <t>מחסני השוק – רד״ק</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.222930,34.802850&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.256575,34.771383&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>31.222930, 34.802850</t>
-        </is>
-      </c>
-      <c r="G63" s="2" t="n"/>
+          <t>31.256575, 34.771383</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="n">
+        <v>1262</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B64" s="2" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי מול</t>
+          <t>מחסני להב ב״ש</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי – מול</t>
+          <t>מחסני להב – באר שבע</t>
         </is>
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.232927,34.797287&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.250485,34.771336&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>31.232927, 34.797287</t>
+          <t>31.250485, 34.771336</t>
         </is>
       </c>
       <c r="G64" s="2" t="n">
-        <v>1231</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="65">
@@ -2422,38 +2424,36 @@
         <v>9</v>
       </c>
       <c r="B65" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>קרפור סינמה סיטי</t>
+          <t>יוחננוף ב״שׁ</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>קרפור – סינמה סיטי באר שבע</t>
+          <t>יוחננוף – באר שבע</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.234304,34.798478&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.241510,34.809600&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>31.234304, 34.798478</t>
-        </is>
-      </c>
-      <c r="G65" s="2" t="n">
-        <v>190</v>
-      </c>
+          <t>31.241510, 34.809600</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
         <v>9</v>
       </c>
       <c r="B66" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="G66" s="2" t="n">
-        <v>765</v>
+        <v>2366</v>
       </c>
     </row>
     <row r="67">
@@ -2484,30 +2484,30 @@
         <v>9</v>
       </c>
       <c r="B67" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>יוחננוף ב״שׁ</t>
+          <t>מחסני השוק שכונה ט</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>יוחננוף – באר שבע</t>
+          <t>מחסני השוק – שכונה ט׳</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.241510,34.809600&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.245847,34.780029&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>31.241510, 34.809600</t>
+          <t>31.245847, 34.780029</t>
         </is>
       </c>
       <c r="G67" s="2" t="n">
-        <v>1519</v>
+        <v>1751</v>
       </c>
     </row>
     <row r="68">
@@ -2515,30 +2515,30 @@
         <v>9</v>
       </c>
       <c r="B68" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי ביג ב״ש</t>
+          <t>קרפור נווה זאב ב״ש</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי – BIG באר שבע</t>
+          <t>קרפור – נווה זאב</t>
         </is>
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.242737,34.813938&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.239300,34.773840&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>31.242737, 34.813938</t>
+          <t>31.239300, 34.773840</t>
         </is>
       </c>
       <c r="G68" s="2" t="n">
-        <v>434</v>
+        <v>1314</v>
       </c>
     </row>
     <row r="69">
@@ -2546,30 +2546,30 @@
         <v>9</v>
       </c>
       <c r="B69" s="2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>טיב טעם ב״ש</t>
+          <t>מחסני השוק יעלים</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>טיב טעם – באר שבע</t>
+          <t>מחסני השוק – יעלים</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.247910,34.812220&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.251100,34.779480&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>31.247910, 34.812220</t>
+          <t>31.251100, 34.779480</t>
         </is>
       </c>
       <c r="G69" s="2" t="n">
-        <v>598</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="70">
@@ -2577,30 +2577,30 @@
         <v>9</v>
       </c>
       <c r="B70" s="2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק האורגים</t>
+          <t>מחסני השוק אופקים</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – האורגים</t>
+          <t>מחסני השוק – אופקים, מבנה</t>
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.254180,34.817730&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.315153,34.624786&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>31.254180, 34.817730</t>
+          <t>31.315153, 34.624786</t>
         </is>
       </c>
       <c r="G70" s="2" t="n">
-        <v>872</v>
+        <v>18695</v>
       </c>
     </row>
     <row r="71">
@@ -2608,30 +2608,30 @@
         <v>9</v>
       </c>
       <c r="B71" s="2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>ח.נ משקאות הסיטונאי</t>
+          <t>רמי לוי אופקים</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>ח.נ משקאות הסיטונאי</t>
+          <t>רמי לוי – אופקים</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.255990,34.816697&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.293210,34.612890&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>31.255990, 34.816697</t>
+          <t>31.293210, 34.612890</t>
         </is>
       </c>
       <c r="G71" s="2" t="n">
-        <v>224</v>
+        <v>4126</v>
       </c>
     </row>
     <row r="72">
@@ -2643,22 +2643,22 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק דימונה</t>
+          <t>מחסני השוק דימונה ממשית</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – דימונה, פרץ סנטר</t>
+          <t>מחסני השוק – דימונה ממשית</t>
         </is>
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.059750,35.020900&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.059192,35.037017&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>31.059750, 35.020900</t>
+          <t>31.059192, 35.037017</t>
         </is>
       </c>
       <c r="G72" s="2" t="n"/>
@@ -2672,26 +2672,26 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק דימונה ממשית</t>
+          <t>מחסני השוק דימונה</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – דימונה ממשית</t>
+          <t>מחסני השוק – דימונה, פרץ סנטר</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.059192,35.037017&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.059750,35.020900&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>31.059192, 35.037017</t>
+          <t>31.059750, 35.020900</t>
         </is>
       </c>
       <c r="G73" s="2" t="n">
-        <v>1536</v>
+        <v>2431</v>
       </c>
     </row>
     <row r="74">
@@ -2703,26 +2703,26 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>קרפור ערד</t>
+          <t>סאלח דבאח ב״ש</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>קרפור – ערד</t>
+          <t>סאלח דבאח – באר שבע</t>
         </is>
       </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.248230,35.201160&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.224450,34.821690&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>31.248230, 35.201160</t>
+          <t>31.224450, 34.821690</t>
         </is>
       </c>
       <c r="G74" s="2" t="n">
-        <v>26188</v>
+        <v>32927</v>
       </c>
     </row>
     <row r="75">
@@ -2734,26 +2734,26 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק ערד</t>
+          <t>קינג סטור ב״ש</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – ערד</t>
+          <t>קינג סטור – באר שבע</t>
         </is>
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.248640,35.199280&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.224680,34.820200&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>31.248640, 35.199280</t>
+          <t>31.224680, 34.820200</t>
         </is>
       </c>
       <c r="G75" s="2" t="n">
-        <v>184</v>
+        <v>543</v>
       </c>
     </row>
     <row r="76">
@@ -2765,26 +2765,26 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק מיתרים</t>
+          <t>קשת טעמים ב״ש</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – מיתרים</t>
+          <t>קשת טעמים – באר שבע</t>
         </is>
       </c>
       <c r="E76" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.374910,35.007250&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.222930,34.802850&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>31.374910, 35.007250</t>
+          <t>31.222930, 34.802850</t>
         </is>
       </c>
       <c r="G76" s="2" t="n">
-        <v>23020</v>
+        <v>2168</v>
       </c>
     </row>
     <row r="77">
@@ -2796,26 +2796,26 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>סאלח דבאח ב״ש</t>
+          <t>רמי לוי מול</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>סאלח דבאח – באר שבע</t>
+          <t>רמי לוי – מול</t>
         </is>
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.224450,34.821690&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.232927,34.797287&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>31.224450, 34.821690</t>
+          <t>31.232927, 34.797287</t>
         </is>
       </c>
       <c r="G77" s="2" t="n">
-        <v>24305</v>
+        <v>1920</v>
       </c>
     </row>
     <row r="78">
@@ -2827,26 +2827,26 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>קינג סטור ב״ש</t>
+          <t>קרפור סינמה סיטי</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>קינג סטור – באר שבע</t>
+          <t>קרפור – סינמה סיטי באר שבע</t>
         </is>
       </c>
       <c r="E78" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.224680,34.820200&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.234304,34.798478&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>31.224680, 34.820200</t>
+          <t>31.234304, 34.798478</t>
         </is>
       </c>
       <c r="G78" s="2" t="n">
-        <v>144</v>
+        <v>1527</v>
       </c>
     </row>
     <row r="79">
@@ -2990,8 +2990,8 @@
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3007,12 +3007,12 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Total distance (m)</t>
+          <t>Total driving distance (m)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Total distance (km)</t>
+          <t>Total driving distance (km)</t>
         </is>
       </c>
     </row>
@@ -3021,13 +3021,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C2" t="n">
-        <v>20632</v>
+        <v>34797</v>
       </c>
       <c r="D2" t="n">
-        <v>20.6</v>
+        <v>34.8</v>
       </c>
     </row>
     <row r="3">
@@ -3035,13 +3035,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C3" t="n">
-        <v>15841</v>
+        <v>26143</v>
       </c>
       <c r="D3" t="n">
-        <v>15.8</v>
+        <v>26.1</v>
       </c>
     </row>
     <row r="4">
@@ -3049,13 +3049,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C4" t="n">
-        <v>6404</v>
+        <v>8888</v>
       </c>
       <c r="D4" t="n">
-        <v>6.4</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="5">
@@ -3063,13 +3063,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C5" t="n">
-        <v>4989</v>
+        <v>37323</v>
       </c>
       <c r="D5" t="n">
-        <v>5</v>
+        <v>37.3</v>
       </c>
     </row>
     <row r="6">
@@ -3077,13 +3077,13 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C6" t="n">
-        <v>20119</v>
+        <v>21442</v>
       </c>
       <c r="D6" t="n">
-        <v>20.1</v>
+        <v>21.4</v>
       </c>
     </row>
     <row r="7">
@@ -3094,10 +3094,10 @@
         <v>7</v>
       </c>
       <c r="C7" t="n">
-        <v>14712</v>
+        <v>41818</v>
       </c>
       <c r="D7" t="n">
-        <v>14.7</v>
+        <v>41.8</v>
       </c>
     </row>
     <row r="8">
@@ -3105,13 +3105,13 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C8" t="n">
-        <v>47130</v>
+        <v>62150</v>
       </c>
       <c r="D8" t="n">
-        <v>47.1</v>
+        <v>62.2</v>
       </c>
     </row>
     <row r="9">
@@ -3119,13 +3119,13 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
+        <v>7</v>
+      </c>
+      <c r="C9" t="n">
+        <v>9033</v>
+      </c>
+      <c r="D9" t="n">
         <v>9</v>
-      </c>
-      <c r="C9" t="n">
-        <v>7566</v>
-      </c>
-      <c r="D9" t="n">
-        <v>7.6</v>
       </c>
     </row>
     <row r="10">
@@ -3133,13 +3133,13 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C10" t="n">
-        <v>5834</v>
+        <v>30616</v>
       </c>
       <c r="D10" t="n">
-        <v>5.8</v>
+        <v>30.6</v>
       </c>
     </row>
     <row r="11">
@@ -3150,10 +3150,10 @@
         <v>7</v>
       </c>
       <c r="C11" t="n">
-        <v>75378</v>
+        <v>41516</v>
       </c>
       <c r="D11" t="n">
-        <v>75.40000000000001</v>
+        <v>41.5</v>
       </c>
     </row>
     <row r="12">
@@ -3174,7 +3174,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Total distance (km)</t>
+          <t>Total driving distance (km)</t>
         </is>
       </c>
     </row>
@@ -3183,7 +3183,7 @@
         <v>9</v>
       </c>
       <c r="B15" t="n">
-        <v>221.4</v>
+        <v>318.7</v>
       </c>
     </row>
     <row r="16">
@@ -3191,7 +3191,7 @@
         <v>10</v>
       </c>
       <c r="B16" t="n">
-        <v>218.6</v>
+        <v>313.7</v>
       </c>
     </row>
     <row r="17">
@@ -3199,7 +3199,7 @@
         <v>11</v>
       </c>
       <c r="B17" t="n">
-        <v>221</v>
+        <v>314.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Route every day as a round trip from the driver's base
Depot (55 Sokolov St, Ramat HaSharon) is now baked into the whole
pipeline: the driving-distance matrix includes it, day clustering
and per-day ordering optimize the full depot->stops->depot loop
(not an open path), and the site shows explicit depot start/end
cards with their own Waze link plus the depot legs on the map.
Because the depot sits far north of the branch network, this shifts
the optimal split toward fewer, larger days (9 days of up to 9 stops
instead of 10) to amortize the round trip.
</commit_message>
<xml_diff>
--- a/branches_with_waze_links_v3_days.xlsx
+++ b/branches_with_waze_links_v3_days.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G80"/>
+  <dimension ref="A1:G89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -491,25 +491,27 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי יבנה</t>
+          <t>רמי לוי לוד</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי – יבנה</t>
+          <t>רמי לוי – לוד</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.885700,34.733740&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.945270,34.892120&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>31.885700, 34.733740</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="n"/>
+          <t>31.945270, 34.892120</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>29570</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -520,26 +522,26 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק יבנה</t>
+          <t>יוחננוף רמלה</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – יבנה</t>
+          <t>יוחננוף – רמלה</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.877970,34.736400&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.937330,34.886180&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>31.877970, 34.736400</t>
+          <t>31.937330, 34.886180</t>
         </is>
       </c>
       <c r="G3" s="2" t="n">
-        <v>1667</v>
+        <v>1178</v>
       </c>
     </row>
     <row r="4">
@@ -551,26 +553,26 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>סופר בונוס יבנה</t>
+          <t>שוק העיר רמלה רחוב דני מס</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>סופר בונוס – יבנה</t>
+          <t>שוק העיר – רמלה, קניון הרמבלס</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.863087,34.739125&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.929320,34.867530&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>31.863087, 34.739125</t>
+          <t>31.929320, 34.867530</t>
         </is>
       </c>
       <c r="G4" s="2" t="n">
-        <v>2490</v>
+        <v>3098</v>
       </c>
     </row>
     <row r="5">
@@ -582,26 +584,26 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>יוחננוף עקרון</t>
+          <t>שוק העיר רמלה רחוב יעקב דורי</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>יוחננוף – קריית עקרון</t>
+          <t>שוק העיר – נאות שמיר, רמלה</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.860190,34.814490&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.929080,34.849320&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>31.860190, 34.814490</t>
+          <t>31.929080, 34.849320</t>
         </is>
       </c>
       <c r="G5" s="2" t="n">
-        <v>10393</v>
+        <v>2418</v>
       </c>
     </row>
     <row r="6">
@@ -632,7 +634,7 @@
         </is>
       </c>
       <c r="G6" s="2" t="n">
-        <v>9561</v>
+        <v>2852</v>
       </c>
     </row>
     <row r="7">
@@ -644,26 +646,26 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>שוק העיר רמלה רחוב יעקב דורי</t>
+          <t>יוחננוף עקרון</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>שוק העיר – נאות שמיר, רמלה</t>
+          <t>יוחננוף – קריית עקרון</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.929080,34.849320&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.860190,34.814490&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>31.929080, 34.849320</t>
+          <t>31.860190, 34.814490</t>
         </is>
       </c>
       <c r="G7" s="2" t="n">
-        <v>4145</v>
+        <v>10176</v>
       </c>
     </row>
     <row r="8">
@@ -675,26 +677,26 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>שוק העיר רמלה רחוב דני מס</t>
+          <t>סופר בונוס יבנה</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>שוק העיר – רמלה, קניון הרמבלס</t>
+          <t>סופר בונוס – יבנה</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.929320,34.867530&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.863087,34.739125&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>31.929320, 34.867530</t>
+          <t>31.863087, 34.739125</t>
         </is>
       </c>
       <c r="G8" s="2" t="n">
-        <v>2370</v>
+        <v>11306</v>
       </c>
     </row>
     <row r="9">
@@ -706,26 +708,26 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>יוחננוף רמלה</t>
+          <t>מחסני השוק יבנה</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>יוחננוף – רמלה</t>
+          <t>מחסני השוק – יבנה</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.937330,34.886180&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.877970,34.736400&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>31.937330, 34.886180</t>
+          <t>31.877970, 34.736400</t>
         </is>
       </c>
       <c r="G9" s="2" t="n">
-        <v>3014</v>
+        <v>3019</v>
       </c>
     </row>
     <row r="10">
@@ -737,86 +739,84 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי לוד</t>
+          <t>רמי לוי יבנה</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי – לוד</t>
+          <t>רמי לוי – יבנה</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.945270,34.892120&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.885700,34.733740&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>31.945270, 34.892120</t>
+          <t>31.885700, 34.733740</t>
         </is>
       </c>
       <c r="G10" s="2" t="n">
-        <v>1155</v>
+        <v>1268</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B11" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>מחסני השוק יד בנימין</t>
-        </is>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr"/>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – יד בנימין</t>
+          <t>בסיס – סוקולוב 55, רמת השרון (חזרה)</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.792720,34.824080&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=32.144199,34.837710&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>31.792720, 34.824080</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="n"/>
+          <t>32.144199, 34.837710</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>35585</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
         <v>2</v>
       </c>
       <c r="B12" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>מחסני הושק יד בנימין</t>
+          <t>רמי לוי אשדוד</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – יד בנימין</t>
+          <t>רמי לוי – אשדוד</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.792720,34.824080&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.814770,34.660040&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>31.792720, 34.824080</t>
+          <t>31.814770, 34.660040</t>
         </is>
       </c>
       <c r="G12" s="2" t="n">
-        <v>0</v>
+        <v>46788</v>
       </c>
     </row>
     <row r="13">
@@ -824,30 +824,30 @@
         <v>2</v>
       </c>
       <c r="B13" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">יוחננוף גדרה </t>
+          <t>קשת טעמים אשדוד</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>יוחננוף – גדרה</t>
+          <t>קשת טעמים – אשדוד</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.797160,34.767740&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.812130,34.661190&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>31.797160, 34.767740</t>
+          <t>31.812130, 34.661190</t>
         </is>
       </c>
       <c r="G13" s="2" t="n">
-        <v>6945</v>
+        <v>692</v>
       </c>
     </row>
     <row r="14">
@@ -855,30 +855,30 @@
         <v>2</v>
       </c>
       <c r="B14" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>הסל שלנו גדרה</t>
+          <t>טיב טעם אשדוד</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>הסל שלנו – גדרה</t>
+          <t>טיב טעם – אשדוד</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.800510,34.783400&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.810210,34.656140&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>31.800510, 34.783400</t>
+          <t>31.810210, 34.656140</t>
         </is>
       </c>
       <c r="G14" s="2" t="n">
-        <v>2514</v>
+        <v>856</v>
       </c>
     </row>
     <row r="15">
@@ -886,30 +886,30 @@
         <v>2</v>
       </c>
       <c r="B15" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>סיטי מרקט סניף שני גדרה</t>
+          <t>קרפור ד רוגזין אשדוד</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>סיטי מרקט – גדרה, סניף צהלה</t>
+          <t>קרפור – אשדוד רובע ד׳</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.800019,34.789253&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.800290,34.641557&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>31.800019, 34.789253</t>
+          <t>31.800290, 34.641557</t>
         </is>
       </c>
       <c r="G15" s="2" t="n">
-        <v>577</v>
+        <v>2538</v>
       </c>
     </row>
     <row r="16">
@@ -917,30 +917,30 @@
         <v>2</v>
       </c>
       <c r="B16" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>סיטי מרקט סניף ראשון גדרה</t>
+          <t>טסה שוקולד רחוב רוגזין אשדוד</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>סיטי מרקט – גדרה, סניף ציונה</t>
+          <t>טסה – רוגוזין, אשדוד  (client 1)</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.804598,34.790889&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.803469,34.642244&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>31.804598, 34.790889</t>
+          <t>31.803469, 34.642244</t>
         </is>
       </c>
       <c r="G16" s="2" t="n">
-        <v>573</v>
+        <v>521</v>
       </c>
     </row>
     <row r="17">
@@ -948,30 +948,30 @@
         <v>2</v>
       </c>
       <c r="B17" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק גדרה</t>
+          <t>טסה שוקולד רחוב רוגזין אשדוד</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – גדרה</t>
+          <t>טסה – רוגוזין, אשדוד  (client 2)</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.803660,34.784850&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.806300,34.643792&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>31.803660, 34.784850</t>
+          <t>31.806300, 34.643792</t>
         </is>
       </c>
       <c r="G17" s="2" t="n">
-        <v>833</v>
+        <v>351</v>
       </c>
     </row>
     <row r="18">
@@ -979,30 +979,30 @@
         <v>2</v>
       </c>
       <c r="B18" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>שפע ברכה גדרה</t>
+          <t>פרש מרקט מחסני להב יבנה</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>שפע ברכה – גדרה</t>
+          <t>מחסני להב / פרשמרקט – יבנה</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.818301,34.775800&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.866399,34.735819&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>31.818301, 34.775800</t>
+          <t>31.866399, 34.735819</t>
         </is>
       </c>
       <c r="G18" s="2" t="n">
-        <v>2289</v>
+        <v>14168</v>
       </c>
     </row>
     <row r="19">
@@ -1010,30 +1010,26 @@
         <v>2</v>
       </c>
       <c r="B19" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>פרש מרקט מחסני להב יבנה</t>
-        </is>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr"/>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>מחסני להב / פרשמרקט – יבנה</t>
+          <t>בסיס – סוקולוב 55, רמת השרון (חזרה)</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.866399,34.735819&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=32.144199,34.837710&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>31.866399, 34.735819</t>
+          <t>32.144199, 34.837710</t>
         </is>
       </c>
       <c r="G19" s="2" t="n">
-        <v>12412</v>
+        <v>36778</v>
       </c>
     </row>
     <row r="20">
@@ -1045,25 +1041,27 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>סופר קופיקס אשדוד</t>
+          <t>מחסני הושק יד בנימין</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>סופר קופיקס – אשדוד</t>
+          <t>מחסני השוק – יד בנימין</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.777726,34.636456&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.792720,34.824080&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>31.777726, 34.636456</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="n"/>
+          <t>31.792720, 34.824080</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>46559</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1074,26 +1072,26 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>זול ובגדול אשדוד</t>
+          <t>מחסני השוק יד בנימין</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>זול ובגדול – אשדוד</t>
+          <t>מחסני השוק – יד בנימין</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.780820,34.631780&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.792720,34.824080&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>31.780820, 34.631780</t>
+          <t>31.792720, 34.824080</t>
         </is>
       </c>
       <c r="G21" s="2" t="n">
-        <v>719</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -1105,26 +1103,26 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>טסה שוקולד רחוב הציונות אשדוד</t>
+          <t>הסל שלנו גדרה</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>טסה – שדרות הציונות, אשדוד</t>
+          <t>הסל שלנו – גדרה</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.787595,34.643303&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.800510,34.783400&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>31.787595, 34.643303</t>
+          <t>31.800510, 34.783400</t>
         </is>
       </c>
       <c r="G22" s="2" t="n">
-        <v>1712</v>
+        <v>5837</v>
       </c>
     </row>
     <row r="23">
@@ -1136,26 +1134,26 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>קרפור ד רוגזין אשדוד</t>
+          <t>סיטי מרקט סניף שני גדרה</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>קרפור – אשדוד רובע ד׳</t>
+          <t>סיטי מרקט – גדרה, סניף צהלה</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.800290,34.641557&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.800019,34.789253&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>31.800290, 34.641557</t>
+          <t>31.800019, 34.789253</t>
         </is>
       </c>
       <c r="G23" s="2" t="n">
-        <v>1822</v>
+        <v>577</v>
       </c>
     </row>
     <row r="24">
@@ -1167,26 +1165,26 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>טסה שוקולד רחוב רוגזין אשדוד</t>
+          <t>סיטי מרקט סניף ראשון גדרה</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>טסה – רוגוזין, אשדוד  (client 1)</t>
+          <t>סיטי מרקט – גדרה, סניף ציונה</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.803469,34.642244&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.804598,34.790889&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>31.803469, 34.642244</t>
+          <t>31.804598, 34.790889</t>
         </is>
       </c>
       <c r="G24" s="2" t="n">
-        <v>521</v>
+        <v>573</v>
       </c>
     </row>
     <row r="25">
@@ -1198,26 +1196,26 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>טסה שוקולד רחוב רוגזין אשדוד</t>
+          <t>מחסני השוק גדרה</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>טסה – רוגוזין, אשדוד  (client 2)</t>
+          <t>מחסני השוק – גדרה</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.806300,34.643792&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.803660,34.784850&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>31.806300, 34.643792</t>
+          <t>31.803660, 34.784850</t>
         </is>
       </c>
       <c r="G25" s="2" t="n">
-        <v>351</v>
+        <v>833</v>
       </c>
     </row>
     <row r="26">
@@ -1229,26 +1227,26 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>טיב טעם אשדוד</t>
+          <t>שפע ברכה גדרה</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>טיב טעם – אשדוד</t>
+          <t>שפע ברכה – גדרה</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.810210,34.656140&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.818301,34.775800&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>31.810210, 34.656140</t>
+          <t>31.818301, 34.775800</t>
         </is>
       </c>
       <c r="G26" s="2" t="n">
-        <v>1843</v>
+        <v>2289</v>
       </c>
     </row>
     <row r="27">
@@ -1260,26 +1258,26 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>קשת טעמים אשדוד</t>
+          <t xml:space="preserve">יוחננוף גדרה </t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>קשת טעמים – אשדוד</t>
+          <t>יוחננוף – גדרה</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.812130,34.661190&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.797160,34.767740&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>31.812130, 34.661190</t>
+          <t>31.797160, 34.767740</t>
         </is>
       </c>
       <c r="G27" s="2" t="n">
-        <v>996</v>
+        <v>4118</v>
       </c>
     </row>
     <row r="28">
@@ -1291,86 +1289,84 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי אשדוד</t>
+          <t>יוחננוף גן יבנה</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי – אשדוד</t>
+          <t>יוחננוף – גן יבנה</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.814770,34.660040&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.794680,34.705580&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>31.814770, 34.660040</t>
+          <t>31.794680, 34.705580</t>
         </is>
       </c>
       <c r="G28" s="2" t="n">
-        <v>924</v>
+        <v>8741</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B29" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>יוחננוף גן יבנה</t>
-        </is>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="C29" s="2" t="inlineStr"/>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>יוחננוף – גן יבנה</t>
+          <t>בסיס – סוקולוב 55, רמת השרון (חזרה)</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.794680,34.705580&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=32.144199,34.837710&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>31.794680, 34.705580</t>
-        </is>
-      </c>
-      <c r="G29" s="2" t="n"/>
+          <t>32.144199, 34.837710</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>47702</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
         <v>4</v>
       </c>
       <c r="B30" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>קרפור ח אשדוד מרכז כלניות</t>
+          <t>פרש מרקט מחסני להב רחוב גיא אוני אשדוד</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>קרפור – אשדוד רובע ח׳, מרכז כלניות</t>
+          <t>מחסני להב / פרשמרקט – גיא אוני</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.783685,34.653253&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.785248,34.659107&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>31.783685, 34.653253</t>
+          <t>31.785248, 34.659107</t>
         </is>
       </c>
       <c r="G30" s="2" t="n">
-        <v>6294</v>
+        <v>49656</v>
       </c>
     </row>
     <row r="31">
@@ -1378,30 +1374,30 @@
         <v>4</v>
       </c>
       <c r="B31" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>פרש מרקט מחסני להב רחוב שהם אשדוד</t>
+          <t>קרפור ח אשדוד מרכז כלניות</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>מחסני להב / פרשמרקט – שוהם</t>
+          <t>קרפור – אשדוד רובע ח׳, מרכז כלניות</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.766695,34.631168&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.783685,34.653253&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>31.766695, 34.631168</t>
+          <t>31.783685, 34.653253</t>
         </is>
       </c>
       <c r="G31" s="2" t="n">
-        <v>3633</v>
+        <v>893</v>
       </c>
     </row>
     <row r="32">
@@ -1409,30 +1405,30 @@
         <v>4</v>
       </c>
       <c r="B32" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>פרש מרקט מחסני להב רחוב גיא אוני אשדוד</t>
+          <t>פרש מרקט מחסני להב רחוב שהם אשדוד</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>מחסני להב / פרשמרקט – גיא אוני</t>
+          <t>מחסני להב / פרשמרקט – שוהם</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.785248,34.659107&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.766695,34.631168&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>31.785248, 34.659107</t>
+          <t>31.766695, 34.631168</t>
         </is>
       </c>
       <c r="G32" s="2" t="n">
-        <v>4259</v>
+        <v>3633</v>
       </c>
     </row>
     <row r="33">
@@ -1440,30 +1436,30 @@
         <v>4</v>
       </c>
       <c r="B33" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>יוחננוף מבקיעים אשקלון</t>
+          <t>סופר קופיקס אשדוד</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>יוחננוף – מבקיעים</t>
+          <t>סופר קופיקס – אשדוד</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.701280,34.579940&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.777726,34.636456&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>31.701280, 34.579940</t>
+          <t>31.777726, 34.636456</t>
         </is>
       </c>
       <c r="G33" s="2" t="n">
-        <v>16150</v>
+        <v>1651</v>
       </c>
     </row>
     <row r="34">
@@ -1471,30 +1467,30 @@
         <v>4</v>
       </c>
       <c r="B34" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>קרפור אפרידר שדרות ירושלים</t>
+          <t>זול ובגדול אשדוד</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>קרפור – אפרידר</t>
+          <t>זול ובגדול – אשדוד</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.677410,34.575410&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.780820,34.631780&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>31.677410, 34.575410</t>
+          <t>31.780820, 34.631780</t>
         </is>
       </c>
       <c r="G34" s="2" t="n">
-        <v>2994</v>
+        <v>719</v>
       </c>
     </row>
     <row r="35">
@@ -1502,30 +1498,30 @@
         <v>4</v>
       </c>
       <c r="B35" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>שוק העיר מכללה אשקלון רחוב אלי כהן</t>
+          <t>טסה שוקולד רחוב הציונות אשדוד</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>שוק העיר – מכללה אשקלון</t>
+          <t>טסה – שדרות הציונות, אשדוד</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.667450,34.569030&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.787595,34.643303&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>31.667450, 34.569030</t>
+          <t>31.787595, 34.643303</t>
         </is>
       </c>
       <c r="G35" s="2" t="n">
-        <v>1716</v>
+        <v>1712</v>
       </c>
     </row>
     <row r="36">
@@ -1533,90 +1529,88 @@
         <v>4</v>
       </c>
       <c r="B36" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>קרפור אשקלון בסיטי קיבוץ גלויות 5</t>
+          <t>יוחננוף מבקיעים אשקלון</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>קרפור – אשקלון סיטי</t>
+          <t>יוחננוף – מבקיעים</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.655189,34.556142&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.701280,34.579940&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>31.655189, 34.556142</t>
+          <t>31.701280, 34.579940</t>
         </is>
       </c>
       <c r="G36" s="2" t="n">
-        <v>2276</v>
+        <v>17108</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B37" s="2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק קרית מלאכי</t>
+          <t>קרפור אפרידר שדרות ירושלים</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – קריית מלאכי</t>
+          <t>קרפור – אפרידר</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.731658,34.753038&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.677410,34.575410&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>31.731658, 34.753038</t>
-        </is>
-      </c>
-      <c r="G37" s="2" t="n"/>
+          <t>31.677410, 34.575410</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="n">
+        <v>2994</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B38" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>מחסני השוק קרית מלאכי</t>
-        </is>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="C38" s="2" t="inlineStr"/>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – קריית מלאכי</t>
+          <t>בסיס – סוקולוב 55, רמת השרון (חזרה)</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.731658,34.753038&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=32.144199,34.837710&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>31.731658, 34.753038</t>
+          <t>32.144199, 34.837710</t>
         </is>
       </c>
       <c r="G38" s="2" t="n">
-        <v>0</v>
+        <v>65271</v>
       </c>
     </row>
     <row r="39">
@@ -1624,30 +1618,30 @@
         <v>5</v>
       </c>
       <c r="B39" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי קסטינה</t>
+          <t>מחסני השוק קרית מלאכי</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי – קסטינה</t>
+          <t>מחסני השוק – קריית מלאכי</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.727796,34.754099&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.731658,34.753038&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>31.727796, 34.754099</t>
+          <t>31.731658, 34.753038</t>
         </is>
       </c>
       <c r="G39" s="2" t="n">
-        <v>1045</v>
+        <v>56547</v>
       </c>
     </row>
     <row r="40">
@@ -1655,30 +1649,30 @@
         <v>5</v>
       </c>
       <c r="B40" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי כרמי גת- בוייז ספורטק קריית גת</t>
+          <t>מחסני השוק קרית מלאכי</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי כרמי גת / סופרמרקט בקריית גת</t>
+          <t>מחסני השוק – קריית מלאכי</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.626950,34.771360&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.731658,34.753038&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>31.626950, 34.771360</t>
+          <t>31.731658, 34.753038</t>
         </is>
       </c>
       <c r="G40" s="2" t="n">
-        <v>16232</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -1686,30 +1680,30 @@
         <v>5</v>
       </c>
       <c r="B41" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>שוק העיר קריית גת- עבודה פרש סוללות ופזים</t>
+          <t>רמי לוי קסטינה</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>שוק העיר – קריית גת / הערת עבודה נוספת</t>
+          <t>רמי לוי – קסטינה</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.604380,34.774310&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.727796,34.754099&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>31.604380, 34.774310</t>
+          <t>31.727796, 34.754099</t>
         </is>
       </c>
       <c r="G41" s="2" t="n">
-        <v>3318</v>
+        <v>1045</v>
       </c>
     </row>
     <row r="42">
@@ -1717,30 +1711,30 @@
         <v>5</v>
       </c>
       <c r="B42" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי קריית גת</t>
+          <t>שוק העיר קריית גת- עבודה פרש סוללות ופזים</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי – קריית גת</t>
+          <t>שוק העיר – קריית גת / הערת עבודה נוספת</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.603820,34.772470&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.604380,34.774310&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>31.603820, 34.772470</t>
+          <t>31.604380, 34.774310</t>
         </is>
       </c>
       <c r="G42" s="2" t="n">
-        <v>293</v>
+        <v>16802</v>
       </c>
     </row>
     <row r="43">
@@ -1748,183 +1742,181 @@
         <v>5</v>
       </c>
       <c r="B43" s="2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק קריית גת</t>
+          <t>רמי לוי קריית גת</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – קריית גת</t>
+          <t>רמי לוי – קריית גת</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.601807,34.772956&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.603820,34.772470&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>31.601807, 34.772956</t>
+          <t>31.603820, 34.772470</t>
         </is>
       </c>
       <c r="G43" s="2" t="n">
-        <v>554</v>
+        <v>293</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B44" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B44" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>יוחננוף נתיבות רחוב אליהו אילוז</t>
+          <t>מחסני השוק קריית גת</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>יוחננוף – נתיבות, אליהו אילוז</t>
+          <t>מחסני השוק – קריית גת</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.412450,34.572680&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.601807,34.772956&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>31.412450, 34.572680</t>
-        </is>
-      </c>
-      <c r="G44" s="2" t="n"/>
+          <t>31.601807, 34.772956</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="n">
+        <v>554</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B45" s="2" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>קרפור נתיבות</t>
+          <t>רמי לוי כרמי גת- בוייז ספורטק קריית גת</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>קרפור – נתיבות</t>
+          <t>רמי לוי כרמי גת / סופרמרקט בקריית גת</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.417980,34.592430&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.626950,34.771360&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>31.417980, 34.592430</t>
+          <t>31.626950, 34.771360</t>
         </is>
       </c>
       <c r="G45" s="2" t="n">
-        <v>2656</v>
+        <v>3820</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B46" s="2" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>יוחננוף נתיבות רחוב בעלי המלאכה</t>
+          <t>רמי לוי אשקלון צפון</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>יוחננוף – נתיבות, בעלי המלאכה</t>
+          <t>רמי לוי – אשקלון צפון</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.418300,34.597040&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.662130,34.594590&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>31.418300, 34.597040</t>
+          <t>31.662130, 34.594590</t>
         </is>
       </c>
       <c r="G46" s="2" t="n">
-        <v>449</v>
+        <v>21258</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B47" s="2" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי נתיבות</t>
+          <t>שוק העיר מכללה אשקלון רחוב אלי כהן</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי – נתיבות</t>
+          <t>שוק העיר – מכללה אשקלון</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.416910,34.615611&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.667450,34.569030&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>31.416910, 34.615611</t>
+          <t>31.667450, 34.569030</t>
         </is>
       </c>
       <c r="G47" s="2" t="n">
-        <v>2710</v>
+        <v>3103</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B48" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>קרפור שדרות</t>
-        </is>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="C48" s="2" t="inlineStr"/>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>קרפור – שדרות</t>
+          <t>בסיס – סוקולוב 55, רמת השרון (חזרה)</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.523700,34.605850&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=32.144199,34.837710&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>31.523700, 34.605850</t>
+          <t>32.144199, 34.837710</t>
         </is>
       </c>
       <c r="G48" s="2" t="n">
-        <v>14390</v>
+        <v>66587</v>
       </c>
     </row>
     <row r="49">
@@ -1932,30 +1924,30 @@
         <v>6</v>
       </c>
       <c r="B49" s="2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי שדרות</t>
+          <t>קרפור אשקלון בסיטי קיבוץ גלויות 5</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי – שדרות</t>
+          <t>קרפור – אשקלון סיטי</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.526502,34.602092&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.655189,34.556142&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>31.526502, 34.602092</t>
+          <t>31.655189, 34.556142</t>
         </is>
       </c>
       <c r="G49" s="2" t="n">
-        <v>904</v>
+        <v>68205</v>
       </c>
     </row>
     <row r="50">
@@ -1963,937 +1955,1208 @@
         <v>6</v>
       </c>
       <c r="B50" s="2" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי אשקלון צפון</t>
+          <t>יוחננוף נתיבות רחוב אליהו אילוז</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי – אשקלון צפון</t>
+          <t>יוחננוף – נתיבות, אליהו אילוז</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.662130,34.594590&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.412450,34.572680&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>31.662130, 34.594590</t>
+          <t>31.412450, 34.572680</t>
         </is>
       </c>
       <c r="G50" s="2" t="n">
-        <v>20709</v>
+        <v>33890</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B51" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי ביג ב״ש</t>
+          <t>קרפור נתיבות</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי – BIG באר שבע</t>
+          <t>קרפור – נתיבות</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.242737,34.813938&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.417980,34.592430&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>31.242737, 34.813938</t>
-        </is>
-      </c>
-      <c r="G51" s="2" t="n"/>
+          <t>31.417980, 34.592430</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="n">
+        <v>2656</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B52" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>טיב טעם ב״ש</t>
+          <t>יוחננוף נתיבות רחוב בעלי המלאכה</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>טיב טעם – באר שבע</t>
+          <t>יוחננוף – נתיבות, בעלי המלאכה</t>
         </is>
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.247910,34.812220&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.418300,34.597040&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>31.247910, 34.812220</t>
+          <t>31.418300, 34.597040</t>
         </is>
       </c>
       <c r="G52" s="2" t="n">
-        <v>920</v>
+        <v>449</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B53" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק האורגים</t>
+          <t>רמי לוי אופקים</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – האורגים</t>
+          <t>רמי לוי – אופקים</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.254180,34.817730&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.293210,34.612890&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>31.254180, 34.817730</t>
+          <t>31.293210, 34.612890</t>
         </is>
       </c>
       <c r="G53" s="2" t="n">
-        <v>1457</v>
+        <v>19887</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B54" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>ח.נ משקאות הסיטונאי</t>
+          <t>מחסני השוק אופקים</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>ח.נ משקאות הסיטונאי</t>
+          <t>מחסני השוק – אופקים, מבנה</t>
         </is>
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.255990,34.816697&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.315153,34.624786&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>31.255990, 34.816697</t>
+          <t>31.315153, 34.624786</t>
         </is>
       </c>
       <c r="G54" s="2" t="n">
-        <v>594</v>
+        <v>4152</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B55" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B55" s="2" t="n">
-        <v>5</v>
-      </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק מיתרים</t>
+          <t>רמי לוי נתיבות</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – מיתרים</t>
+          <t>רמי לוי – נתיבות</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.374910,35.007250&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.416910,34.615611&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>31.374910, 35.007250</t>
+          <t>31.416910, 34.615611</t>
         </is>
       </c>
       <c r="G55" s="2" t="n">
-        <v>24366</v>
+        <v>16084</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B56" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>קרפור ערד</t>
+          <t>קרפור שדרות</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>קרפור – ערד</t>
+          <t>קרפור – שדרות</t>
         </is>
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.248230,35.201160&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.523700,34.605850&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>31.248230, 35.201160</t>
+          <t>31.523700, 34.605850</t>
         </is>
       </c>
       <c r="G56" s="2" t="n">
-        <v>34289</v>
+        <v>14390</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B57" s="2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק ערד</t>
+          <t>רמי לוי שדרות</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – ערד</t>
+          <t>רמי לוי – שדרות</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.248640,35.199280&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.526502,34.602092&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>31.248640, 35.199280</t>
+          <t>31.526502, 34.602092</t>
         </is>
       </c>
       <c r="G57" s="2" t="n">
-        <v>525</v>
+        <v>904</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B58" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C58" s="2" t="inlineStr">
-        <is>
-          <t>מחסני השוק רמות</t>
-        </is>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="C58" s="2" t="inlineStr"/>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – רמות</t>
+          <t>בסיס – סוקולוב 55, רמת השרון (חזרה)</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.280323,34.804813&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=32.144199,34.837710&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>31.280323, 34.804813</t>
-        </is>
-      </c>
-      <c r="G58" s="2" t="n"/>
+          <t>32.144199, 34.837710</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="n">
+        <v>83630</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B59" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>קרפור צפון ב״ש רחוב אברהם אבינו</t>
+          <t>מחסני השוק הקריה החרדית</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>קרפור – באר שבע, שכונה ד׳</t>
+          <t>מחסני השוק מהדרין – הקריה החרדית</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.270018,34.797222&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.267940,34.778430&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>31.270018, 34.797222</t>
+          <t>31.267940, 34.778430</t>
         </is>
       </c>
       <c r="G59" s="2" t="n">
-        <v>2412</v>
+        <v>107594</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B60" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק הקריה החרדית</t>
+          <t>קרפור קניון אביה</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק מהדרין – הקריה החרדית</t>
+          <t>קרפור – קניון אביה</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.267940,34.778430&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.263278,34.778719&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>31.267940, 34.778430</t>
+          <t>31.263278, 34.778719</t>
         </is>
       </c>
       <c r="G60" s="2" t="n">
-        <v>2175</v>
+        <v>927</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B61" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>קרפור קניון אביה</t>
+          <t>מחסני השוק רד״ק</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>קרפור – קניון אביה</t>
+          <t>מחסני השוק – רד״ק</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.263278,34.778719&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.256575,34.771383&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>31.263278, 34.778719</t>
+          <t>31.256575, 34.771383</t>
         </is>
       </c>
       <c r="G61" s="2" t="n">
-        <v>927</v>
+        <v>1434</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B62" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק עובדה</t>
+          <t>מחסני להב ב״ש</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – עובדה</t>
+          <t>מחסני להב – באר שבע</t>
         </is>
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.259650,34.780120&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.250485,34.771336&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>31.259650, 34.780120</t>
+          <t>31.250485, 34.771336</t>
         </is>
       </c>
       <c r="G62" s="2" t="n">
-        <v>948</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B63" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק רד״ק</t>
+          <t>קרפור נווה זאב ב״ש</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – רד״ק</t>
+          <t>קרפור – נווה זאב</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.256575,34.771383&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.239300,34.773840&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>31.256575, 34.771383</t>
+          <t>31.239300, 34.773840</t>
         </is>
       </c>
       <c r="G63" s="2" t="n">
-        <v>1262</v>
+        <v>2650</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B64" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>מחסני להב ב״ש</t>
+          <t>מחסני השוק יעלים</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>מחסני להב – באר שבע</t>
+          <t>מחסני השוק – יעלים</t>
         </is>
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.250485,34.771336&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.251100,34.779480&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>31.250485, 34.771336</t>
+          <t>31.251100, 34.779480</t>
         </is>
       </c>
       <c r="G64" s="2" t="n">
-        <v>1309</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B65" s="2" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>יוחננוף ב״שׁ</t>
+          <t>מחסני השוק עובדה</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>יוחננוף – באר שבע</t>
+          <t>מחסני השוק – עובדה</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.241510,34.809600&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.259650,34.780120&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>31.241510, 34.809600</t>
-        </is>
-      </c>
-      <c r="G65" s="2" t="n"/>
+          <t>31.259650, 34.780120</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="n">
+        <v>1771</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B66" s="2" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק בית אשל</t>
+          <t>קרפור צפון ב״ש רחוב אברהם אבינו</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – בית אשל</t>
+          <t>קרפור – באר שבע, שכונה ד׳</t>
         </is>
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.239870,34.793740&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.270018,34.797222&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>31.239870, 34.793740</t>
+          <t>31.270018, 34.797222</t>
         </is>
       </c>
       <c r="G66" s="2" t="n">
-        <v>2366</v>
+        <v>2830</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B67" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="B67" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="C67" s="2" t="inlineStr">
-        <is>
-          <t>מחסני השוק שכונה ט</t>
-        </is>
-      </c>
+      <c r="C67" s="2" t="inlineStr"/>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – שכונה ט׳</t>
+          <t>בסיס – סוקולוב 55, רמת השרון (חזרה)</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.245847,34.780029&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=32.144199,34.837710&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>31.245847, 34.780029</t>
+          <t>32.144199, 34.837710</t>
         </is>
       </c>
       <c r="G67" s="2" t="n">
-        <v>1751</v>
+        <v>106555</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B68" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>קרפור נווה זאב ב״ש</t>
+          <t>מחסני השוק בית אשל</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>קרפור – נווה זאב</t>
+          <t>מחסני השוק – בית אשל</t>
         </is>
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.239300,34.773840&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.239870,34.793740&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>31.239300, 34.773840</t>
+          <t>31.239870, 34.793740</t>
         </is>
       </c>
       <c r="G68" s="2" t="n">
-        <v>1314</v>
+        <v>109945</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B69" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק יעלים</t>
+          <t>יוחננוף ב״שׁ</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – יעלים</t>
+          <t>יוחננוף – באר שבע</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.251100,34.779480&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.241510,34.809600&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>31.251100, 34.779480</t>
+          <t>31.241510, 34.809600</t>
         </is>
       </c>
       <c r="G69" s="2" t="n">
-        <v>2364</v>
+        <v>2573</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B70" s="2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק אופקים</t>
+          <t>טיב טעם ב״ש</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – אופקים, מבנה</t>
+          <t>טיב טעם – באר שבע</t>
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.315153,34.624786&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.247910,34.812220&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>31.315153, 34.624786</t>
+          <t>31.247910, 34.812220</t>
         </is>
       </c>
       <c r="G70" s="2" t="n">
-        <v>18695</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B71" s="2" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי אופקים</t>
+          <t>קרפור סינמה סיטי</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי – אופקים</t>
+          <t>קרפור – סינמה סיטי באר שבע</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.293210,34.612890&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.234304,34.798478&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>31.293210, 34.612890</t>
+          <t>31.234304, 34.798478</t>
         </is>
       </c>
       <c r="G71" s="2" t="n">
-        <v>4126</v>
+        <v>2722</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B72" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק דימונה ממשית</t>
+          <t>סאלח דבאח ב״ש</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – דימונה ממשית</t>
+          <t>סאלח דבאח – באר שבע</t>
         </is>
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.059192,35.037017&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.224450,34.821690&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>31.059192, 35.037017</t>
-        </is>
-      </c>
-      <c r="G72" s="2" t="n"/>
+          <t>31.224450, 34.821690</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="n">
+        <v>2950</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B73" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק דימונה</t>
+          <t>קינג סטור ב״ש</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>מחסני השוק – דימונה, פרץ סנטר</t>
+          <t>קינג סטור – באר שבע</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.059750,35.020900&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.224680,34.820200&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>31.059750, 35.020900</t>
+          <t>31.224680, 34.820200</t>
         </is>
       </c>
       <c r="G73" s="2" t="n">
-        <v>2431</v>
+        <v>543</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B74" s="2" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>סאלח דבאח ב״ש</t>
+          <t>קשת טעמים ב״ש</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>סאלח דבאח – באר שבע</t>
+          <t>קשת טעמים – באר שבע</t>
         </is>
       </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.224450,34.821690&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.222930,34.802850&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>31.224450, 34.821690</t>
+          <t>31.222930, 34.802850</t>
         </is>
       </c>
       <c r="G74" s="2" t="n">
-        <v>32927</v>
+        <v>2168</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B75" s="2" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>קינג סטור ב״ש</t>
+          <t>רמי לוי מול</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>קינג סטור – באר שבע</t>
+          <t>רמי לוי – מול</t>
         </is>
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.224680,34.820200&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.232927,34.797287&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>31.224680, 34.820200</t>
+          <t>31.232927, 34.797287</t>
         </is>
       </c>
       <c r="G75" s="2" t="n">
-        <v>543</v>
+        <v>1920</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B76" s="2" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>קשת טעמים ב״ש</t>
+          <t>מחסני השוק שכונה ט</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>קשת טעמים – באר שבע</t>
+          <t>מחסני השוק – שכונה ט׳</t>
         </is>
       </c>
       <c r="E76" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.222930,34.802850&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=31.245847,34.780029&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>31.222930, 34.802850</t>
+          <t>31.245847, 34.780029</t>
         </is>
       </c>
       <c r="G76" s="2" t="n">
-        <v>2168</v>
+        <v>2414</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B77" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="B77" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="C77" s="2" t="inlineStr">
-        <is>
-          <t>רמי לוי מול</t>
-        </is>
-      </c>
+      <c r="C77" s="2" t="inlineStr"/>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>רמי לוי – מול</t>
+          <t>בסיס – סוקולוב 55, רמת השרון (חזרה)</t>
         </is>
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>https://waze.com/ul?ll=31.232927,34.797287&amp;navigate=yes</t>
+          <t>https://waze.com/ul?ll=32.144199,34.837710&amp;navigate=yes</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>31.232927, 34.797287</t>
+          <t>32.144199, 34.837710</t>
         </is>
       </c>
       <c r="G77" s="2" t="n">
-        <v>1920</v>
+        <v>110448</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B78" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>מחסני השוק רמות</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>מחסני השוק – רמות</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>https://waze.com/ul?ll=31.280323,34.804813&amp;navigate=yes</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>31.280323, 34.804813</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="n">
+        <v>105950</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B79" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>ח.נ משקאות הסיטונאי</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>ח.נ משקאות הסיטונאי</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="inlineStr">
+        <is>
+          <t>https://waze.com/ul?ll=31.255990,34.816697&amp;navigate=yes</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>31.255990, 34.816697</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="n">
+        <v>4846</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B80" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>מחסני השוק האורגים</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>מחסני השוק – האורגים</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="inlineStr">
+        <is>
+          <t>https://waze.com/ul?ll=31.254180,34.817730&amp;navigate=yes</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>31.254180, 34.817730</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="n">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B81" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>רמי לוי ביג ב״ש</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>רמי לוי – BIG באר שבע</t>
+        </is>
+      </c>
+      <c r="E81" s="3" t="inlineStr">
+        <is>
+          <t>https://waze.com/ul?ll=31.242737,34.813938&amp;navigate=yes</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>31.242737, 34.813938</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="n">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B82" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>מחסני השוק דימונה</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>מחסני השוק – דימונה, פרץ סנטר</t>
+        </is>
+      </c>
+      <c r="E82" s="3" t="inlineStr">
+        <is>
+          <t>https://waze.com/ul?ll=31.059750,35.020900&amp;navigate=yes</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>31.059750, 35.020900</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="n">
+        <v>38199</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B83" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>מחסני השוק דימונה ממשית</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>מחסני השוק – דימונה ממשית</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="inlineStr">
+        <is>
+          <t>https://waze.com/ul?ll=31.059192,35.037017&amp;navigate=yes</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>31.059192, 35.037017</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="n">
+        <v>2383</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B84" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>קרפור ערד</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>קרפור – ערד</t>
+        </is>
+      </c>
+      <c r="E84" s="3" t="inlineStr">
+        <is>
+          <t>https://waze.com/ul?ll=31.248230,35.201160&amp;navigate=yes</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>31.248230, 35.201160</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="n">
+        <v>43569</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B85" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>מחסני השוק ערד</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>מחסני השוק – ערד</t>
+        </is>
+      </c>
+      <c r="E85" s="3" t="inlineStr">
+        <is>
+          <t>https://waze.com/ul?ll=31.248640,35.199280&amp;navigate=yes</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>31.248640, 35.199280</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="n">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B86" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>מחסני השוק מיתרים</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>מחסני השוק – מיתרים</t>
+        </is>
+      </c>
+      <c r="E86" s="3" t="inlineStr">
+        <is>
+          <t>https://waze.com/ul?ll=31.374910,35.007250&amp;navigate=yes</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>31.374910, 35.007250</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="n">
+        <v>33984</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B87" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="B78" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="C78" s="2" t="inlineStr">
-        <is>
-          <t>קרפור סינמה סיטי</t>
-        </is>
-      </c>
-      <c r="D78" s="2" t="inlineStr">
-        <is>
-          <t>קרפור – סינמה סיטי באר שבע</t>
-        </is>
-      </c>
-      <c r="E78" s="3" t="inlineStr">
-        <is>
-          <t>https://waze.com/ul?ll=31.234304,34.798478&amp;navigate=yes</t>
-        </is>
-      </c>
-      <c r="F78" s="2" t="inlineStr">
-        <is>
-          <t>31.234304, 34.798478</t>
-        </is>
-      </c>
-      <c r="G78" s="2" t="n">
-        <v>1527</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="2" t="inlineStr">
+      <c r="C87" s="2" t="inlineStr"/>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>בסיס – סוקולוב 55, רמת השרון (חזרה)</t>
+        </is>
+      </c>
+      <c r="E87" s="3" t="inlineStr">
+        <is>
+          <t>https://waze.com/ul?ll=32.144199,34.837710&amp;navigate=yes</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>32.144199, 34.837710</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="n">
+        <v>120917</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
         <is>
           <t>Unscheduled</t>
         </is>
       </c>
-      <c r="B79" s="2" t="n"/>
-      <c r="C79" s="2" t="inlineStr">
+      <c r="B88" s="2" t="n"/>
+      <c r="C88" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">קרפור לב אשקלון </t>
         </is>
       </c>
-      <c r="D79" s="2" t="inlineStr">
+      <c r="D88" s="2" t="inlineStr">
         <is>
           <t>קרפור – לב אשקלון</t>
         </is>
       </c>
-      <c r="E79" s="2" t="inlineStr"/>
-      <c r="F79" s="2" t="inlineStr"/>
-      <c r="G79" s="2" t="n"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="2" t="inlineStr">
+      <c r="E88" s="2" t="inlineStr"/>
+      <c r="F88" s="2" t="inlineStr"/>
+      <c r="G88" s="2" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
         <is>
           <t>Unscheduled</t>
         </is>
       </c>
-      <c r="B80" s="2" t="n"/>
-      <c r="C80" s="2" t="inlineStr">
+      <c r="B89" s="2" t="n"/>
+      <c r="C89" s="2" t="inlineStr">
         <is>
           <t>מחסני השוק סניף חדש</t>
         </is>
       </c>
-      <c r="D80" s="2" t="inlineStr">
+      <c r="D89" s="2" t="inlineStr">
         <is>
           <t>מחסני השוק – סניף חדש</t>
         </is>
       </c>
-      <c r="E80" s="2" t="inlineStr">
+      <c r="E89" s="2" t="inlineStr">
         <is>
           <t>TODO</t>
         </is>
       </c>
-      <c r="F80" s="2" t="inlineStr"/>
-      <c r="G80" s="2" t="n"/>
+      <c r="F89" s="2" t="inlineStr"/>
+      <c r="G89" s="2" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -2974,6 +3237,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E76" r:id="rId75"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E77" r:id="rId76"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E78" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E79" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E80" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E81" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E82" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E83" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E84" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E85" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E86" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E87" r:id="rId86"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2985,11 +3257,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
   </cols>
@@ -3007,7 +3279,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Total driving distance (m)</t>
+          <t>Total driving distance (m, incl. depot round trip)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -3024,10 +3296,10 @@
         <v>9</v>
       </c>
       <c r="C2" t="n">
-        <v>34797</v>
+        <v>100471</v>
       </c>
       <c r="D2" t="n">
-        <v>34.8</v>
+        <v>100.5</v>
       </c>
     </row>
     <row r="3">
@@ -3035,13 +3307,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C3" t="n">
-        <v>26143</v>
+        <v>102693</v>
       </c>
       <c r="D3" t="n">
-        <v>26.1</v>
+        <v>102.7</v>
       </c>
     </row>
     <row r="4">
@@ -3052,10 +3324,10 @@
         <v>9</v>
       </c>
       <c r="C4" t="n">
-        <v>8888</v>
+        <v>117229</v>
       </c>
       <c r="D4" t="n">
-        <v>8.9</v>
+        <v>117.2</v>
       </c>
     </row>
     <row r="5">
@@ -3066,10 +3338,10 @@
         <v>8</v>
       </c>
       <c r="C5" t="n">
-        <v>37323</v>
+        <v>143638</v>
       </c>
       <c r="D5" t="n">
-        <v>37.3</v>
+        <v>143.6</v>
       </c>
     </row>
     <row r="6">
@@ -3077,13 +3349,13 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C6" t="n">
-        <v>21442</v>
+        <v>170008</v>
       </c>
       <c r="D6" t="n">
-        <v>21.4</v>
+        <v>170</v>
       </c>
     </row>
     <row r="7">
@@ -3091,13 +3363,13 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C7" t="n">
-        <v>41818</v>
+        <v>244249</v>
       </c>
       <c r="D7" t="n">
-        <v>41.8</v>
+        <v>244.2</v>
       </c>
     </row>
     <row r="8">
@@ -3105,13 +3377,13 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C8" t="n">
-        <v>62150</v>
+        <v>227433</v>
       </c>
       <c r="D8" t="n">
-        <v>62.2</v>
+        <v>227.4</v>
       </c>
     </row>
     <row r="9">
@@ -3119,13 +3391,13 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C9" t="n">
-        <v>9033</v>
+        <v>236838</v>
       </c>
       <c r="D9" t="n">
-        <v>9</v>
+        <v>236.8</v>
       </c>
     </row>
     <row r="10">
@@ -3133,73 +3405,71 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C10" t="n">
-        <v>30616</v>
+        <v>352847</v>
       </c>
       <c r="D10" t="n">
-        <v>30.6</v>
+        <v>352.8</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
-        <v>10</v>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Unscheduled</t>
+        </is>
       </c>
       <c r="B11" t="n">
-        <v>7</v>
-      </c>
-      <c r="C11" t="n">
-        <v>41516</v>
-      </c>
-      <c r="D11" t="n">
-        <v>41.5</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Unscheduled</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Depot: בסיס – סוקולוב 55, רמת השרון</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>32.144199, 34.837710</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Day-count option</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Total driving distance (km)</t>
         </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>9</v>
-      </c>
-      <c r="B15" t="n">
-        <v>318.7</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B16" t="n">
-        <v>313.7</v>
+        <v>1695.4</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
+        <v>10</v>
+      </c>
+      <c r="B17" t="n">
+        <v>1825.9</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
         <v>11</v>
       </c>
-      <c r="B17" t="n">
-        <v>314.8</v>
+      <c r="B18" t="n">
+        <v>2016.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>